<commit_message>
feat: must reduction optimizer e melhorias gerais
</commit_message>
<xml_diff>
--- a/dados/11 - Envision.xlsx
+++ b/dados/11 - Envision.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Debian\home\cver\projects\solar-bess-modulation-risk\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C076064-0346-4CF8-B396-4215B456E6EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03944584-B8D8-459D-8E8E-209303857654}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11175" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{0BE0756F-E6AA-4360-A796-BF3CFC3D6C24}"/>
   </bookViews>
@@ -57,7 +57,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -83,14 +90,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -422,7 +432,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75426E42-EE39-42D5-B014-625E751B77C6}">
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -733,6 +743,176 @@
         <v>0.8431018590927124</v>
       </c>
     </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>21</v>
+      </c>
+      <c r="B23" s="1">
+        <f>(1-(B21-B22)/B21)*B22</f>
+        <v>0.69242748202809135</v>
+      </c>
+      <c r="C23" s="1">
+        <f>(1-(C21-C22)/C21)*C22</f>
+        <v>0.93675011580090239</v>
+      </c>
+      <c r="D23" s="1">
+        <f>(1-(D21-D22)/D21)*D22</f>
+        <v>0.84227279967682533</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>22</v>
+      </c>
+      <c r="B24" s="1">
+        <f>(1-(B22-B23)/B22)*B23</f>
+        <v>0.68350987578134936</v>
+      </c>
+      <c r="C24" s="1">
+        <f t="shared" ref="C24:D24" si="0">(1-(C22-C23)/C22)*C23</f>
+        <v>0.93651027036823786</v>
+      </c>
+      <c r="D24" s="1">
+        <f t="shared" si="0"/>
+        <v>0.84144455551179753</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>23</v>
+      </c>
+      <c r="B25" s="1">
+        <f>(1-(B23-B24)/B23)*B24</f>
+        <v>0.67470711723091636</v>
+      </c>
+      <c r="C25" s="1">
+        <f t="shared" ref="C25:D25" si="1">(1-(C23-C24)/C23)*C24</f>
+        <v>0.93627048634558074</v>
+      </c>
+      <c r="D25" s="1">
+        <f t="shared" si="1"/>
+        <v>0.84061712579595671</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>24</v>
+      </c>
+      <c r="B26" s="1">
+        <f>(1-(B24-B25)/B24)*B25</f>
+        <v>0.66601772728105935</v>
+      </c>
+      <c r="C26" s="1">
+        <f t="shared" ref="C26:D26" si="2">(1-(C24-C25)/C24)*C25</f>
+        <v>0.93603076371720761</v>
+      </c>
+      <c r="D26" s="1">
+        <f t="shared" si="2"/>
+        <v>0.83979050972841895</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>25</v>
+      </c>
+      <c r="B27" s="1">
+        <f>(1-(B25-B26)/B25)*B26</f>
+        <v>0.65744024588496208</v>
+      </c>
+      <c r="C27" s="1">
+        <f t="shared" ref="C27:D27" si="3">(1-(C25-C26)/C25)*C26</f>
+        <v>0.93579110246739916</v>
+      </c>
+      <c r="D27" s="1">
+        <f t="shared" si="3"/>
+        <v>0.83896470650908772</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>26</v>
+      </c>
+      <c r="B28" s="1">
+        <f>(1-(B26-B27)/B26)*B27</f>
+        <v>0.64897323179939836</v>
+      </c>
+      <c r="C28" s="1">
+        <f t="shared" ref="C28:D28" si="4">(1-(C26-C27)/C26)*C27</f>
+        <v>0.93555150258043995</v>
+      </c>
+      <c r="D28" s="1">
+        <f t="shared" si="4"/>
+        <v>0.83813971533865339</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>27</v>
+      </c>
+      <c r="B29" s="1">
+        <f>(1-(B27-B28)/B27)*B28</f>
+        <v>0.64061526234256538</v>
+      </c>
+      <c r="C29" s="1">
+        <f t="shared" ref="C29:D29" si="5">(1-(C27-C28)/C27)*C28</f>
+        <v>0.93531196404061867</v>
+      </c>
+      <c r="D29" s="1">
+        <f t="shared" si="5"/>
+        <v>0.83731553541859227</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>28</v>
+      </c>
+      <c r="B30" s="1">
+        <f>(1-(B28-B29)/B28)*B29</f>
+        <v>0.6323649331550355</v>
+      </c>
+      <c r="C30" s="1">
+        <f t="shared" ref="C30:D30" si="6">(1-(C28-C29)/C28)*C29</f>
+        <v>0.93507248683222799</v>
+      </c>
+      <c r="D30" s="1">
+        <f t="shared" si="6"/>
+        <v>0.83649216595116593</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>29</v>
+      </c>
+      <c r="B31" s="1">
+        <f>(1-(B29-B30)/B29)*B30</f>
+        <v>0.62422085796378679</v>
+      </c>
+      <c r="C31" s="1">
+        <f t="shared" ref="C31:D31" si="7">(1-(C29-C30)/C29)*C30</f>
+        <v>0.93483307093956469</v>
+      </c>
+      <c r="D31" s="1">
+        <f t="shared" si="7"/>
+        <v>0.83566960613942043</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>30</v>
+      </c>
+      <c r="B32" s="1">
+        <f>(1-(B30-B31)/B30)*B31</f>
+        <v>0.61618166834927268</v>
+      </c>
+      <c r="C32" s="1">
+        <f t="shared" ref="C32:D32" si="8">(1-(C30-C31)/C30)*C31</f>
+        <v>0.93459371634692945</v>
+      </c>
+      <c r="D32" s="1">
+        <f t="shared" si="8"/>
+        <v>0.83484785518718541</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>